<commit_message>
Catálogo: leer INE del apoderado y boleta del Registro Público
- Nuevos tipos de documento en "Llenar desde PDF" y "Alta desde PDFs":
  boleta del RPP (folio, fecha y lugar de inscripción) e INE (identificación
  y vigencia del apoderado; CURP y sexo en personas físicas).
- La INE se une al apoderado con ese nombre; si no existe, a la empresa del
  nombre del archivo como apoderado nuevo. El nombre del archivo también
  sirve para ubicar la empresa de poderes, actas y boletas.
- Apoderado con INE y vigencia (aviso si venció), variable
  identificacion_representante y dos columnas al final del Excel.
- La IA (servidor) reconoce y lee los dos tipos nuevos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UwdpqyTuNpXdq3bY8FzPVX
</commit_message>
<xml_diff>
--- a/catalogo/catalogo-partes-plantilla.xlsx
+++ b/catalogo/catalogo-partes-plantilla.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="49">
   <si>
     <t>Tipo (Moral/Física)</t>
   </si>
@@ -112,6 +112,12 @@
   </si>
   <si>
     <t>Sexo (persona física)</t>
+  </si>
+  <si>
+    <t>INE del apoderado</t>
+  </si>
+  <si>
+    <t>Vigencia INE del apoderado (año)</t>
   </si>
   <si>
     <t>Empresa (RFC o razón social)</t>
@@ -568,7 +574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AJ500"/>
+  <dimension ref="A1:AL500"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="14" customWidth="1"/>
@@ -603,9 +609,11 @@
     <col min="34" max="34" width="10" customWidth="1"/>
     <col min="35" max="35" width="40" customWidth="1"/>
     <col min="36" max="36" width="12" customWidth="1"/>
+    <col min="37" max="37" width="36" customWidth="1"/>
+    <col min="38" max="38" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:38" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -713,6 +721,12 @@
       </c>
       <c r="AJ1" s="3" t="s">
         <v>32</v>
+      </c>
+      <c r="AK1" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="AL1" s="5" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:34" x14ac:dyDescent="0.25"/>
@@ -1253,16 +1267,16 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1281,52 +1295,52 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>